<commit_message>
fix: mejorar deteccion de sabores en el excel
</commit_message>
<xml_diff>
--- a/lista_precios_clientes.xlsx
+++ b/lista_precios_clientes.xlsx
@@ -421,7 +421,7 @@
         <v>Star Nutrition Whey Platinum 2lb Doy Pack</v>
       </c>
       <c r="C2" t="str">
-        <v>Único</v>
+        <v>Chocolate</v>
       </c>
       <c r="D2">
         <v>69900</v>
@@ -533,7 +533,7 @@
         <v>Whey Protein 907 gr - BODY ADVANCE Frutos Rojos</v>
       </c>
       <c r="C10" t="str">
-        <v>Único</v>
+        <v>Frutos Rojos</v>
       </c>
       <c r="D10">
         <v>42900</v>
@@ -547,7 +547,7 @@
         <v>Vegetal Protein Isolate 2 lbs coco - GOLD NUTRITION</v>
       </c>
       <c r="C11" t="str">
-        <v>Único</v>
+        <v>Coco</v>
       </c>
       <c r="D11">
         <v>40900</v>
@@ -561,7 +561,7 @@
         <v>Creatina Micronized Neutro 200gr - ONE FIT</v>
       </c>
       <c r="C12" t="str">
-        <v>Único</v>
+        <v>Neutro</v>
       </c>
       <c r="D12">
         <v>14900</v>
@@ -617,7 +617,7 @@
         <v>OPTIMUS Collagen Sabor Naranja 240gr - ONE FIT</v>
       </c>
       <c r="C16" t="str">
-        <v>Único</v>
+        <v>Naranja</v>
       </c>
       <c r="D16">
         <v>16900</v>

</xml_diff>

<commit_message>
fix: assign new photos and improve smart flavor detection
</commit_message>
<xml_diff>
--- a/lista_precios_clientes.xlsx
+++ b/lista_precios_clientes.xlsx
@@ -435,7 +435,7 @@
         <v>Star Nutrition TNT Dynamite 240gr</v>
       </c>
       <c r="C3" t="str">
-        <v>Único</v>
+        <v>Sin Sabor</v>
       </c>
       <c r="D3">
         <v>28900</v>
@@ -477,7 +477,7 @@
         <v>Star Nutrition Caffeine 200 x30 Caps</v>
       </c>
       <c r="C6" t="str">
-        <v>Único</v>
+        <v>Sin Sabor (Cápsulas)</v>
       </c>
       <c r="D6">
         <v>9900</v>
@@ -491,7 +491,7 @@
         <v>Xtrenght Nutrition Shaker Espiral 600ml</v>
       </c>
       <c r="C7" t="str">
-        <v>Único</v>
+        <v>N/A</v>
       </c>
       <c r="D7">
         <v>9900</v>
@@ -505,7 +505,7 @@
         <v>Citrato de Magnesio 150g 60 serv. - ONE FIT</v>
       </c>
       <c r="C8" t="str">
-        <v>Único</v>
+        <v>Sin Sabor</v>
       </c>
       <c r="D8">
         <v>7900</v>
@@ -519,7 +519,7 @@
         <v>Omega 3 - 30 caps - ONE FIT NUTRITION</v>
       </c>
       <c r="C9" t="str">
-        <v>Único</v>
+        <v>Sin Sabor (Cápsulas)</v>
       </c>
       <c r="D9">
         <v>24900</v>
@@ -561,7 +561,7 @@
         <v>Creatina Micronized Neutro 200gr - ONE FIT</v>
       </c>
       <c r="C12" t="str">
-        <v>Neutro</v>
+        <v>Neutra, Neutro</v>
       </c>
       <c r="D12">
         <v>14900</v>
@@ -575,7 +575,7 @@
         <v>Creatina Monohidratada 500g - ONE FIT</v>
       </c>
       <c r="C13" t="str">
-        <v>Único</v>
+        <v>Neutra</v>
       </c>
       <c r="D13">
         <v>31900</v>
@@ -603,7 +603,7 @@
         <v>Creatina Monohidrato EEUU 300g - ENA</v>
       </c>
       <c r="C15" t="str">
-        <v>Único</v>
+        <v>Neutra</v>
       </c>
       <c r="D15">
         <v>29900</v>

</xml_diff>

<commit_message>
feat: agregar Colageno Star Nutrition, Citrato de Magnesio XBODY y ajustar precio Creatina Gold a 27900
</commit_message>
<xml_diff>
--- a/lista_precios_clientes.xlsx
+++ b/lista_precios_clientes.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -424,7 +424,7 @@
         <v>Chocolate</v>
       </c>
       <c r="D2">
-        <v>69900</v>
+        <v>73900</v>
       </c>
     </row>
     <row r="3">
@@ -449,7 +449,7 @@
         <v>Creatina Monohidrato 300g - Star Nutrition</v>
       </c>
       <c r="C4" t="str">
-        <v>Sin Sabor (Doypack), Fruit Punch (Doypack), Neutra (Pote)</v>
+        <v>Sin Sabor (Doypack), Fruit Punch (Doypack)</v>
       </c>
       <c r="D4">
         <v>28900</v>
@@ -463,7 +463,7 @@
         <v>Creatina Micronizada 300gr - ENA</v>
       </c>
       <c r="C5" t="str">
-        <v>Sin Sabor, Fruit Punch</v>
+        <v>Sin Sabor, Fruit Punch, Naranja</v>
       </c>
       <c r="D5">
         <v>29900</v>
@@ -477,7 +477,7 @@
         <v>Star Nutrition Caffeine 200 x30 Caps</v>
       </c>
       <c r="C6" t="str">
-        <v>Sin Sabor (Cápsulas)</v>
+        <v>Único</v>
       </c>
       <c r="D6">
         <v>9900</v>
@@ -491,7 +491,7 @@
         <v>Xtrenght Nutrition Shaker Espiral 600ml</v>
       </c>
       <c r="C7" t="str">
-        <v>N/A</v>
+        <v>Único</v>
       </c>
       <c r="D7">
         <v>9900</v>
@@ -505,7 +505,7 @@
         <v>Citrato de Magnesio 150g 60 serv. - ONE FIT</v>
       </c>
       <c r="C8" t="str">
-        <v>Sin Sabor</v>
+        <v>Único</v>
       </c>
       <c r="D8">
         <v>7900</v>
@@ -519,7 +519,7 @@
         <v>Omega 3 - 30 caps - ONE FIT NUTRITION</v>
       </c>
       <c r="C9" t="str">
-        <v>Sin Sabor (Cápsulas)</v>
+        <v>Único</v>
       </c>
       <c r="D9">
         <v>24900</v>
@@ -530,13 +530,13 @@
         <v>BODY ADVANCE</v>
       </c>
       <c r="B10" t="str">
-        <v>Whey Protein 907 gr - BODY ADVANCE Frutos Rojos</v>
+        <v>Whey Protein 907 gr - BODY ADVANCE</v>
       </c>
       <c r="C10" t="str">
-        <v>Frutos Rojos</v>
+        <v>Frutos Rojos, Chocolate</v>
       </c>
       <c r="D10">
-        <v>42900</v>
+        <v>40900</v>
       </c>
     </row>
     <row r="11">
@@ -575,7 +575,7 @@
         <v>Creatina Monohidratada 500g - ONE FIT</v>
       </c>
       <c r="C13" t="str">
-        <v>Neutra</v>
+        <v>Único</v>
       </c>
       <c r="D13">
         <v>31900</v>
@@ -603,7 +603,7 @@
         <v>Creatina Monohidrato EEUU 300g - ENA</v>
       </c>
       <c r="C15" t="str">
-        <v>Neutra</v>
+        <v>Único</v>
       </c>
       <c r="D15">
         <v>29900</v>
@@ -623,9 +623,65 @@
         <v>17900</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Star Nutrition</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Creatina Monohidrato 300g Pote - Star Nutrition</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Neutra</v>
+      </c>
+      <c r="D17">
+        <v>30900</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>GOLD NUTRITION</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Creatina Monohidrato 300g - GOLD NUTRITION</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Único</v>
+      </c>
+      <c r="D18">
+        <v>27900</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Star Nutrition</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Star Nutrition Collagen 210g Sabor Limón</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Limón</v>
+      </c>
+      <c r="D19">
+        <v>18900</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>XBODY Evolution</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Citrato de Magnesio 120 Cápsulas - XBODY Evolution</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Único</v>
+      </c>
+      <c r="D20">
+        <v>14900</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>